<commit_message>
Drop the two 1.7L 'quiet' jugs from compact-kettles sheet
Remove Russell Hobbs Quiet Boil 20462 and Breville Edge VKT236 at the user's
request: both are full-size 1.7L, not compact, and no genuinely compact RH or
Breville kettle is sold in the allowed IE stores. Sheet now has 5 products;
Method sheet documents the removal.
</commit_message>
<xml_diff>
--- a/research/compact-kettles-ireland.xlsx
+++ b/research/compact-kettles-ireland.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="22" customWidth="1" min="18" max="18"/>
@@ -798,56 +798,56 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Russell Hobbs Quiet Boil 20462 (1.7L)</t>
+          <t>Tefal Includeo KI533840 (1L)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Russell Hobbs</t>
+          <t>Tefal</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Standard jug</t>
+          <t>Compact standard</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>No (1.7L — substitute; no compact RH sold in IE)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1.7</v>
+        <v>1</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>6.8</v>
+        <v>4</v>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>1 cup / 235 ml (per claim); window MIN marking needs verification</t>
+          <t>1 cup / 0.3 L (markings 0.3/0.5/0.7/1.0 L)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Yes (claim: 1 cup in 45 s)</t>
+          <t>Yes (0.3 L)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>23.8 × 16.2 × 22.8 cm (snippet — needs verification)</t>
+          <t>16.6 × 20.0 × 23.2 cm (W×D×H)</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>23.8 × 16.2</t>
+          <t>16.6 × 20.0</t>
         </is>
       </c>
       <c r="L3" s="2" t="n">
-        <v>385.6</v>
+        <v>332</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
@@ -860,11 +860,11 @@
         </is>
       </c>
       <c r="O3" s="2" t="n">
-        <v>3000</v>
+        <v>2400</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>1 cup (235 ml) in 45 s (not full-boil time)</t>
+          <t>1 L from cold in 3 min 07 s (187 s) — full boil, published</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>"up to 75% quieter" (no dB published)</t>
+          <t>needs verification</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -894,46 +894,46 @@
       </c>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Plastic w/ brushed-steel finish (needs verification)</t>
+          <t>Plastic</t>
         </is>
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>2 years (snippet — needs verification)</t>
+          <t>2 years</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>Currys.ie; Harvey Norman.ie</t>
+          <t>needs verification (not confirmed on the 4 allowed stores; only Tefal IE shop)</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>needs verification (live IE € not retrievable; UK £34.99 not usable)</t>
+          <t>needs verification on allowed store (Tefal IE shop €61.00, 2026-06-15, not an allowed source)</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>Per-cup only: 3000W×45s = 0.0375 kWh → €0.014 (from 45 s claim); full-boil needs verification</t>
+          <t>Full 1 L: 2400W×187s = 0.1247 kWh → €0.045</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.1867</v>
+        <v>0.1098</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>0.0678</v>
+        <v>0.0399</v>
       </c>
       <c r="AC3" s="2" t="n">
         <v>0.01</v>
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>Awin (Currys.ie / HN.ie)</t>
+          <t>needs verification (no allowed IE retailer confirmed)</t>
         </is>
       </c>
       <c r="AE3" s="2" t="inlineStr">
         <is>
-          <t>No compact (sub-1.7L) non-travel RH sold in the 4 IE stores; this is RH's quiet option. Recommend reviewing — see Method sheet.</t>
+          <t>Genuinely compact 1L and boils 1 cup; but not confirmed in the 4 allowed IE stores — verify stock/price on HN.ie or Amazon.ie.</t>
         </is>
       </c>
     </row>
@@ -943,52 +943,52 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Breville Edge Low Steam VKT236 (1.7L)</t>
+          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Breville</t>
+          <t>Philips</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Standard jug</t>
+          <t>Standard jug (smallest Philips in IE)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>No (1.7L — no compact Breville sold in IE)</t>
+          <t>Borderline (1.5L; no travel/mini Philips in IE)</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1.7</v>
+        <v>1.5</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>6.8</v>
+        <v>6</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>~250 ml / 1 cup actual; lowest window marking 2 cups (manual/review — needs verification)</t>
+          <t>needs verification</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Yes (1 cup, unmarked)</t>
+          <t>needs verification</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>16.2 × 21.5 × 26.2 cm (Currys snippet — needs verification)</t>
+          <t>22.3 × 16.2 × 25.4 cm</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>16.2 × 21.5</t>
+          <t>22.3 × 16.2</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
-        <v>348.3</v>
+        <v>361.3</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
@@ -1001,11 +1001,11 @@
         </is>
       </c>
       <c r="O4" s="2" t="n">
-        <v>3000</v>
+        <v>2200</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>needs verification (mfr); review: 1 L in 2 min 29 s</t>
+          <t>needs verification</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -1015,81 +1015,81 @@
       </c>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>needs verification (220–240V expected)</t>
+          <t>220–240V</t>
         </is>
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
+          <t>Yes (micro-mesh &gt;180 µm)</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="T4" s="2" t="inlineStr">
-        <is>
-          <t>"Quiet Mark approved – 50% quieter boil" (no mfr dB; review 56 dB)</t>
-        </is>
-      </c>
-      <c r="U4" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="V4" s="2" t="inlineStr">
         <is>
-          <t>Stainless steel</t>
+          <t>Plastic (PP) + concealed steel element</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>1 year (Currys; mfr needs verification — some list 2)</t>
+          <t>2 years (variant needs verification)</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>Currys.ie; Amazon.ie</t>
+          <t>Currys.ie (HN.ie stocks Philips; this model not confirmed)</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>Currys.ie €69.99 (snippet, 2026-06-15, needs verification live); Amazon.ie ~€64.62 (snippet)</t>
+          <t>needs verification on allowed store (ref ~€39 at non-allowed source, 2026-06-15)</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>needs verification (no full-boil time published)</t>
+          <t>needs verification (no boil time published)</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.1867</v>
+        <v>0.1647</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>0.0678</v>
+        <v>0.0598</v>
       </c>
       <c r="AC4" s="2" t="n">
         <v>0.01</v>
       </c>
       <c r="AD4" s="2" t="inlineStr">
         <is>
-          <t>Awin (Currys.ie); Amazon Associates (Amazon.ie)</t>
+          <t>Awin (Currys.ie)</t>
         </is>
       </c>
       <c r="AE4" s="2" t="inlineStr">
         <is>
-          <t>Breville's only quiet option in IE; the true compact 1L (BKE320/395) is Australia-only. Recommend reviewing — see Method sheet.</t>
+          <t>Smallest Philips in IE but still 1.5L full-size. Kept pending your call on whether to drop it too (it is NOT a 'quiet' model).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Tefal Includeo KI533840 (1L)</t>
+          <t>Dualit 1 Litre Jug Kettle 72200 (1L)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Tefal</t>
+          <t>Dualit</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1110,26 +1110,26 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>1 cup / 0.3 L (markings 0.3/0.5/0.7/1.0 L)</t>
+          <t>2 cups (manufacturer minimum)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Yes (0.3 L)</t>
+          <t>No (min 2 cups)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>16.6 × 20.0 × 23.2 cm (W×D×H)</t>
+          <t>20 × 16 × 23 cm (weight 0.92 kg)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>16.6 × 20.0</t>
+          <t>20 × 16</t>
         </is>
       </c>
       <c r="L5" s="2" t="n">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
@@ -1141,12 +1141,14 @@
           <t>needs verification</t>
         </is>
       </c>
-      <c r="O5" s="2" t="n">
-        <v>2400</v>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (1L 72200 not stated; only the 1.5L 'Lite' is 3 kW — do not assume)</t>
+        </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>1 L from cold in 3 min 07 s (187 s) — full boil, published</t>
+          <t>needs verification</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -1156,7 +1158,7 @@
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>needs verification (220–240V expected)</t>
+          <t>needs verification (220–240V implied)</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
@@ -1166,7 +1168,7 @@
       </c>
       <c r="T5" s="2" t="inlineStr">
         <is>
-          <t>needs verification</t>
+          <t>needs verification (no quiet-boil claim on the 1L model; Dualit markets the Classic as quiet, not this)</t>
         </is>
       </c>
       <c r="U5" s="2" t="inlineStr">
@@ -1176,27 +1178,27 @@
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>Plastic</t>
+          <t>Stainless steel</t>
         </is>
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>2 years</t>
+          <t>1 year (mfr; some retailers list 2–3)</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>needs verification (not confirmed on the 4 allowed stores; only Tefal IE shop)</t>
+          <t>Currys.ie (Dualit category page confirmed; exact 72200 product/price/stock needs verification)</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>needs verification on allowed store (Tefal IE shop €61.00, 2026-06-15, not an allowed source)</t>
+          <t>needs verification (Currys.ie / Amazon.ie not retrievable; 72200 not found in Amazon.ie search)</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>Full 1 L: 2400W×187s = 0.1247 kWh → €0.045</t>
+          <t>needs verification (no boil time and no confirmed wattage)</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
@@ -1210,48 +1212,48 @@
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>needs verification (no allowed IE retailer confirmed)</t>
+          <t>Awin (Currys.ie)</t>
         </is>
       </c>
       <c r="AE5" s="2" t="inlineStr">
         <is>
-          <t>Genuinely compact 1L and boils 1 cup; but not confirmed in the 4 allowed IE stores — verify stock/price on HN.ie or Amazon.ie.</t>
+          <t>Chosen over Salter (Salter has no compact model in IE). Genuinely compact 1L; min boil is 2 cups, not 1. NB: 'Lite' range is a separate 1.5L line — don't confuse 72200 (1L) with Lite 72003/06/10/12 (1.5L).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
+          <t>Kenwood Discovery JKP250 (0.5L)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Philips</t>
+          <t>Kenwood</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Standard jug (smallest Philips in IE)</t>
+          <t>Travel / mini</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Borderline (1.5L; no travel/mini Philips in IE)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>needs verification</t>
+          <t>NV (ships with 2×200 ml cups; MIN marking not confirmed)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1261,29 +1263,29 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>22.3 × 16.2 × 25.4 cm</t>
+          <t>16.8 × 9.8 × 17.0 cm (W×D×H)</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>22.3 × 16.2</t>
+          <t>16.8 × 9.8</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
-        <v>361.3</v>
+        <v>164.6</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>needs verification</t>
+          <t>N/A (corded travel — no separate base)</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>needs verification</t>
+          <t>16.8 × 9.8 (kettle only)</t>
         </is>
       </c>
       <c r="O6" s="2" t="n">
-        <v>2200</v>
+        <v>650</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -1292,17 +1294,17 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>Cordless</t>
+          <t>Corded</t>
         </is>
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>220–240V</t>
+          <t>Dual / universal 120–240V</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>Yes (micro-mesh &gt;180 µm)</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="T6" s="2" t="inlineStr">
@@ -1317,22 +1319,22 @@
       </c>
       <c r="V6" s="2" t="inlineStr">
         <is>
-          <t>Plastic (PP) + concealed steel element</t>
+          <t>Plastic</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>2 years (variant needs verification)</t>
+          <t>1 year</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>Currys.ie (HN.ie stocks Philips; this model not confirmed)</t>
+          <t>Currys.ie (listed)</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>needs verification on allowed store (ref ~€39 at non-allowed source, 2026-06-15)</t>
+          <t>needs verification (listed on Currys.ie; € not retrievable, 2026-06-15)</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr">
@@ -1341,10 +1343,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.1647</v>
+        <v>0.0549</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>0.0598</v>
+        <v>0.0199</v>
       </c>
       <c r="AC6" s="2" t="n">
         <v>0.01</v>
@@ -1355,290 +1357,6 @@
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
-        <is>
-          <t>Smallest Philips in IE but still 1.5L full-size. Recommend reviewing — see Method sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Dualit 1 Litre Jug Kettle 72200 (1L)</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Dualit</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Compact standard</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>2 cups (manufacturer minimum)</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>No (min 2 cups)</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>20 × 16 × 23 cm (weight 0.92 kg)</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>20 × 16</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="n">
-        <v>320</v>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>needs verification</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>needs verification</t>
-        </is>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>needs verification (1L 72200 not stated; only the 1.5L 'Lite' is 3 kW — do not assume)</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
-        <is>
-          <t>needs verification</t>
-        </is>
-      </c>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>Cordless</t>
-        </is>
-      </c>
-      <c r="R7" s="2" t="inlineStr">
-        <is>
-          <t>needs verification (220–240V implied)</t>
-        </is>
-      </c>
-      <c r="S7" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="T7" s="2" t="inlineStr">
-        <is>
-          <t>needs verification (no quiet-boil claim on the 1L model; Dualit markets the Classic as quiet, not this)</t>
-        </is>
-      </c>
-      <c r="U7" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="V7" s="2" t="inlineStr">
-        <is>
-          <t>Stainless steel</t>
-        </is>
-      </c>
-      <c r="W7" s="2" t="inlineStr">
-        <is>
-          <t>1 year (mfr; some retailers list 2–3)</t>
-        </is>
-      </c>
-      <c r="X7" s="2" t="inlineStr">
-        <is>
-          <t>Currys.ie (Dualit category page confirmed; exact 72200 product/price/stock needs verification)</t>
-        </is>
-      </c>
-      <c r="Y7" s="2" t="inlineStr">
-        <is>
-          <t>needs verification (Currys.ie / Amazon.ie not retrievable; 72200 not found in Amazon.ie search)</t>
-        </is>
-      </c>
-      <c r="Z7" s="2" t="inlineStr">
-        <is>
-          <t>needs verification (no boil time and no confirmed wattage)</t>
-        </is>
-      </c>
-      <c r="AA7" s="2" t="n">
-        <v>0.1098</v>
-      </c>
-      <c r="AB7" s="2" t="n">
-        <v>0.0399</v>
-      </c>
-      <c r="AC7" s="2" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="AD7" s="2" t="inlineStr">
-        <is>
-          <t>Awin (Currys.ie)</t>
-        </is>
-      </c>
-      <c r="AE7" s="2" t="inlineStr">
-        <is>
-          <t>Chosen over Salter (Salter has no compact model in IE). Genuinely compact 1L; min boil is 2 cups, not 1. NB: 'Lite' range is a separate 1.5L line — don't confuse 72200 (1L) with Lite 72003/06/10/12 (1.5L).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Kenwood Discovery JKP250 (0.5L)</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Kenwood</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Travel / mini</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>NV (ships with 2×200 ml cups; MIN marking not confirmed)</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>needs verification</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>16.8 × 9.8 × 17.0 cm (W×D×H)</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>16.8 × 9.8</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="n">
-        <v>164.6</v>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>N/A (corded travel — no separate base)</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>16.8 × 9.8 (kettle only)</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>650</v>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>needs verification</t>
-        </is>
-      </c>
-      <c r="Q8" s="2" t="inlineStr">
-        <is>
-          <t>Corded</t>
-        </is>
-      </c>
-      <c r="R8" s="2" t="inlineStr">
-        <is>
-          <t>Dual / universal 120–240V</t>
-        </is>
-      </c>
-      <c r="S8" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="T8" s="2" t="inlineStr">
-        <is>
-          <t>needs verification</t>
-        </is>
-      </c>
-      <c r="U8" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>Plastic</t>
-        </is>
-      </c>
-      <c r="W8" s="2" t="inlineStr">
-        <is>
-          <t>1 year</t>
-        </is>
-      </c>
-      <c r="X8" s="2" t="inlineStr">
-        <is>
-          <t>Currys.ie (listed)</t>
-        </is>
-      </c>
-      <c r="Y8" s="2" t="inlineStr">
-        <is>
-          <t>needs verification (listed on Currys.ie; € not retrievable, 2026-06-15)</t>
-        </is>
-      </c>
-      <c r="Z8" s="2" t="inlineStr">
-        <is>
-          <t>needs verification (no boil time published)</t>
-        </is>
-      </c>
-      <c r="AA8" s="2" t="n">
-        <v>0.0549</v>
-      </c>
-      <c r="AB8" s="2" t="n">
-        <v>0.0199</v>
-      </c>
-      <c r="AC8" s="2" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="AD8" s="2" t="inlineStr">
-        <is>
-          <t>Awin (Currys.ie)</t>
-        </is>
-      </c>
-      <c r="AE8" s="2" t="inlineStr">
         <is>
           <t>Chosen over Tower T10026 (not confirmed in allowed IE stores). Smallest footprint; 2nd travel/mini pick.</t>
         </is>
@@ -1655,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1751,355 +1469,219 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Russell Hobbs Quiet Boil 20462 (1.7L)</t>
+          <t>Tefal Includeo KI533840 (1L)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Specs (power, noise claim, filter, boil claim)</t>
+          <t>Specs (capacity, power, filter, cordless)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://uk.russellhobbs.com/black-quiet-boil-kettle-20462</t>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Russell Hobbs Quiet Boil 20462 (1.7L)</t>
+          <t>Tefal Includeo KI533840 (1L)</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>IE listing / window</t>
+          <t>Min boil markings / boil time / window / warranty</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>https://www.currys.ie/products/russell-hobbs-quiet-boil-20462-jug-kettle-black-10226936.html</t>
+          <t>https://shop.tefal.co.uk/ie/includeo-ki533840-kettle-1l-black</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Russell Hobbs Quiet Boil 20462 (1.7L)</t>
+          <t>Tefal Includeo KI533840 (1L)</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>IE listing / capacity / warranty</t>
+          <t>Dimensions / material (mfr-supplied Amazon spec)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://www.harveynorman.ie/small-appliances/kettles-and-toasters/kettles/russell-hobbs-1.7l-quiet-boil-kettle-20462-black.html</t>
+          <t>https://www.amazon.co.uk/Tefal-KI533840-Includeo-Electric-Capacity/dp/B0B795TDNH</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Breville Edge Low Steam VKT236 (1.7L)</t>
+          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Specs (power, capacity, noise, filter, material)</t>
+          <t>IE listing</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>https://www.breville.co.uk/kettles-and-toasters/kettles/breville-edge-low-steam-kettle-1.7l/VKT236.html</t>
+          <t>https://www.currys.ie/ieen/household-appliances/small-kitchen-appliances/kettles/philips-daily-collection-hd9334-12-jug-kettle-white-blue-10164709-pdt.html</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Breville Edge Low Steam VKT236 (1.7L)</t>
+          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Dimensions / warranty (Currys UK snippet)</t>
+          <t>Specs (capacity, power, voltage) — datasheet mirror</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://www.currys.co.uk/products/breville-edge-low-steam-vkt236-traditional-kettle--brushed-stainless-steel-10258885.html</t>
+          <t>https://icecat.biz/en/p/philips/hd9334-90/daily+collection-electric+kettles-8710103809654-hd9334-90-35700663.html</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Breville Edge Low Steam VKT236 (1.7L)</t>
+          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>IE listing / price</t>
+          <t>Dimensions (Philips datasheet PDF)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>https://www.currys.ie/products/breville-edge-low-steam-vkt236-traditional-kettle--brushed-stainless-steel-10258885.html</t>
+          <t>https://gzhls.at/blob/ldb/b/3/4/5/f7e120e5116fc98814833e52b29d019eee9b.pdf</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Breville Edge Low Steam VKT236 (1.7L)</t>
+          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>IE listing (Amazon)</t>
+          <t>Filter / cordless / window / material</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.ie/Breville-efficient-Brushed-Stainless-VKT236/dp/B0C64N5RM7</t>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Breville Edge Low Steam VKT236 (1.7L)</t>
+          <t>Dualit 1 Litre Jug Kettle 72200 (1L)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Min boil / boil time / dB (independent review — not mfr)</t>
+          <t>Specs (capacity, min boil, dims, filter, material, warranty)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>https://www.expertreviews.co.uk/home-garden/kitchen/breville-edge-low-steam-kettle-review</t>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Tefal Includeo KI533840 (1L)</t>
+          <t>Dualit 1 Litre Jug Kettle 72200 (1L)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Specs (capacity, power, filter, cordless)</t>
+          <t>Model number 72200</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+          <t>https://www.hartsofstur.com/dualit-1-litre-mini-jug-kettle-chrome-72200.html</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Tefal Includeo KI533840 (1L)</t>
+          <t>Dualit 1 Litre Jug Kettle 72200 (1L)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Min boil markings / boil time / window / warranty</t>
+          <t>IE category page</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tefal.co.uk/ie/includeo-ki533840-kettle-1l-black</t>
+          <t>https://www.currys.ie/appliances/small-kitchen-appliances/kettles/dualit</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Tefal Includeo KI533840 (1L)</t>
+          <t>Kenwood Discovery JKP250 (0.5L)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Dimensions / material (mfr-supplied Amazon spec)</t>
+          <t>Specs (capacity, power, voltage, filter, window, material, warranty)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.co.uk/Tefal-KI533840-Includeo-Electric-Capacity/dp/B0B795TDNH</t>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
+          <t>Kenwood Discovery JKP250 (0.5L)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>IE listing</t>
+          <t>IE listing (Currys kettle category)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>https://www.currys.ie/ieen/household-appliances/small-kitchen-appliances/kettles/philips-daily-collection-hd9334-12-jug-kettle-white-blue-10164709-pdt.html</t>
+          <t>https://www.currys.ie/appliances/small-kitchen-appliances/kettles/kenwood</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
+          <t>Kenwood Discovery JKP250 (0.5L)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Specs (capacity, power, voltage) — datasheet mirror</t>
+          <t>Dimensions (UK retailer quoting Kenwood — verify)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>https://icecat.biz/en/p/philips/hd9334-90/daily+collection-electric+kettles-8710103809654-hd9334-90-35700663.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Dimensions (Philips datasheet PDF)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>https://gzhls.at/blob/ldb/b/3/4/5/f7e120e5116fc98814833e52b29d019eee9b.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Filter / cordless / window / material</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Dualit 1L Mini Lite Jug Kettle 72200</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Specs (capacity, power, min boil, dims, filter, material, warranty)</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Dualit 1L Mini Lite Jug Kettle 72200</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Model number 72200</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>https://www.hartsofstur.com/dualit-1-litre-mini-jug-kettle-chrome-72200.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Dualit 1L Mini Lite Jug Kettle 72200</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>IE quiet-kettle category</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>https://www.currys.ie/appliances/small-kitchen-appliances/kettles/dualit/quiet-kettles</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Kenwood Discovery JKP250 (0.5L)</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Specs (capacity, power, voltage, filter, window, material, warranty)</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Kenwood Discovery JKP250 (0.5L)</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>IE listing (Currys kettle category)</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>https://www.currys.ie/appliances/small-kitchen-appliances/kettles/kenwood</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Kenwood Discovery JKP250 (0.5L)</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Dimensions (UK retailer quoting Kenwood — verify)</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>https://maxwellselectrical.co.uk/kenwood-jkp250-100023951.html</t>
         </is>
@@ -2116,7 +1698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2132,7 +1714,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Compiled 2026-06-15. One row per product on the 'Kettles' sheet; source URLs on 'Sources'.</t>
+          <t>Compiled 2026-06-15. 5 products (the two 1.7L 'quiet' jugs were dropped — see below). Rows on 'Kettles'; URLs on 'Sources'.</t>
         </is>
       </c>
     </row>
@@ -2163,7 +1745,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>• No marketing prose — factual numbers/claims only. Manufacturer claim text is quoted verbatim where used (e.g. noise).</t>
+          <t>• No marketing prose — factual numbers/claims only. Manufacturer claim text is quoted verbatim where used.</t>
         </is>
       </c>
     </row>
@@ -2280,7 +1862,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Confirmed full-boil time only for Tefal Includeo (1 L in 3:07 → €0.045). RH 20462 publishes a per-cup 45 s claim only.</t>
+          <t xml:space="preserve">  Confirmed full-boil time only for Tefal Includeo (1 L in 3:07 → €0.045).</t>
         </is>
       </c>
     </row>
@@ -2309,96 +1891,99 @@
       <c r="A30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>PRODUCT SUBSTITUTIONS &amp; FLAGS (told to the user)</t>
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>REMOVED AT USER REQUEST</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>• Russell Hobbs compact/quiet: NO compact (sub-1.7L) non-travel RH is sold in the 4 allowed IE stores. The true</t>
+          <t>• Russell Hobbs Quiet Boil 20462 (1.7L) and Breville Edge VKT236 (1.7L) — both full-size 'quiet' jugs, NOT compact.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  compacts (Compact Home 0.8L 24190/24191; Victory Compact 1L 24990) are not on IE retailers. Row uses the Quiet Boil</t>
+          <t xml:space="preserve">  No genuinely compact RH or Breville kettle is sold in the 4 allowed IE stores, so the 'compact quiet' niche was</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  20462 (1.7L, NOT compact) as RH's quiet option — recommend replacing or relabelling.</t>
+          <t xml:space="preserve">  dropped rather than padded with 1.7L models.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>• Breville: NO compact Breville in IE (the 1L BKE320/395 is Australia-only). Row uses the Edge VKT236 (1.7L, NOT compact).</t>
-        </is>
-      </c>
+      <c r="A35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>• Philips: NO travel/mini Philips in IE; whole range is 1.5–1.7L. Row uses the smallest (Daily HD9334/12, 1.5L, borderline).</t>
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>REMAINING PRODUCT FLAGS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>• Dualit chosen over Salter (Salter has no compact model in IE). Dualit 72200 is genuinely compact (1L) but min boil = 2 cups.</t>
+          <t>• Philips: NO travel/mini Philips in IE; whole range is 1.5–1.7L. Row uses the smallest (Daily HD9334/12, 1.5L,</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>• Kenwood JKP250 chosen over Tower T10026 (Tower not confirmed in allowed IE stores).</t>
+          <t xml:space="preserve">  borderline). It is NOT a 'quiet' model, so it was kept — say the word to drop it too.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>• Tefal Includeo KI533840 is genuinely compact (1L, boils 1 cup) but was NOT confirmed in the 4 allowed stores</t>
+          <t>• Dualit chosen over Salter (Salter has no compact model in IE). Dualit 72200 is genuinely compact (1L); min boil = 2 cups.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (only the Tefal IE manufacturer shop) — verify stock/price on HN.ie or Amazon.ie before using.</t>
+          <t>• Kenwood JKP250 chosen over Tower T10026 (Tower not confirmed in allowed IE stores).</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr"/>
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>• Tefal Includeo KI533840 is genuinely compact (1L, boils 1 cup) but was NOT confirmed in the 4 allowed stores</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>NET RESULT: genuinely compact + confirmed in an allowed IE store = RH 23840 (travel), Kenwood JKP250 (travel),</t>
+          <t xml:space="preserve">  (only the Tefal IE manufacturer shop) — verify stock/price on HN.ie or Amazon.ie before using.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Dualit 72200 (compact, Currys quiet category). The 'quiet compact' niche barely exists in the IE market — worth</t>
-        </is>
-      </c>
+      <c r="A43" s="4" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>deciding whether the article covers compact AND 'quiet 1.7L' as separate buckets, or drops the non-compact rows.</t>
+          <t>NET: genuinely compact + confirmed in an allowed IE store today = RH 23840 (travel), Kenwood JKP250 (travel),</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Dualit 72200 (compact). Tefal (compact) and Philips (borderline) need an allowed-store price/stock confirmation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add per-datum source/status sheet to compact-kettles spreadsheet
Replace the grouped 'Sources' sheet with a tidy 'Data & sources' sheet: one row
per (product, field) with value, status (confirmed / needs verification /
calculated / estimate / inference) and the source URL side by side, so every
data point sits next to its source. Method sheet now spells out the footprint
state per product (only Kenwood has a complete kettle+base total).
</commit_message>
<xml_diff>
--- a/research/compact-kettles-ireland.xlsx
+++ b/research/compact-kettles-ireland.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Kettles" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sources" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Data &amp; sources" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Method &amp; notes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,10 @@
     <font>
       <b val="1"/>
       <color rgb="000F172A"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00B7791F"/>
     </font>
     <font>
       <b val="1"/>
@@ -76,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -84,7 +88,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1074,7 +1081,7 @@
       </c>
       <c r="AE4" s="2" t="inlineStr">
         <is>
-          <t>Smallest Philips in IE but still 1.5L full-size. Kept pending your call on whether to drop it too (it is NOT a 'quiet' model).</t>
+          <t>Smallest Philips in IE but still 1.5L full-size; kept as the higher-capacity option (not a 'quiet' model).</t>
         </is>
       </c>
     </row>
@@ -1217,7 +1224,7 @@
       </c>
       <c r="AE5" s="2" t="inlineStr">
         <is>
-          <t>Chosen over Salter (Salter has no compact model in IE). Genuinely compact 1L; min boil is 2 cups, not 1. NB: 'Lite' range is a separate 1.5L line — don't confuse 72200 (1L) with Lite 72003/06/10/12 (1.5L).</t>
+          <t>Chosen over Salter (Salter has no compact model in IE). Genuinely compact 1L; min boil 2 cups. NB: 'Lite' is a separate 1.5L line — don't confuse 72200 (1L) with Lite 72003/06/10/12 (1.5L).</t>
         </is>
       </c>
     </row>
@@ -1373,26 +1380,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Field(s)</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Source URL</t>
         </is>
@@ -1401,15 +1420,25 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Russell Hobbs Compact Travel Kettle 23840 (0.85L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Specs (capacity, power, voltage, filter, warranty, window)</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Travel / mini</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
@@ -1418,272 +1447,3417 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Russell Hobbs Compact Travel Kettle 23840 (0.85L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Capacity / in-stock / price</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.amazon.ie/Russell-Hobbs-23840-Compact-Electric/dp/B07B96BQM6</t>
+          <t>Capacity (L)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Russell Hobbs Compact Travel Kettle 23840 (0.85L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>In-stock IE / warranty</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.harveynorman.ie/small-appliances/kettles-and-toasters/kettles/russell-hobbs-0.85l-compact-travel-kettle-23840-white.html</t>
+          <t>Cups per boil</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>— (derived: capacity ÷ 0.25 L)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Russell Hobbs Compact Travel Kettle 23840 (0.85L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>In-stock IE</t>
+          <t>Min boil</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>https://www.soundstore.ie/small-appliances/small-kitchen-appliances/russell-hobbs-travel-kettle-23840.html</t>
+          <t>NV (ships with 2 cups; MIN marking not confirmed)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Tefal Includeo KI533840 (1L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Specs (capacity, power, filter, cordless)</t>
+          <t>Can boil 1 cup?</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Tefal Includeo KI533840 (1L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Min boil markings / boil time / window / warranty</t>
+          <t>Kettle dims L×D×H (cm)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>https://shop.tefal.co.uk/ie/includeo-ki533840-kettle-1l-black</t>
+          <t>H 18.1 cm; L×D needs verification</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>partly confirmed — see value</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Tefal Includeo KI533840 (1L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Dimensions / material (mfr-supplied Amazon spec)</t>
+          <t>Kettle footprint L×D (cm)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>https://www.amazon.co.uk/Tefal-KI533840-Includeo-Electric-Capacity/dp/B0B795TDNH</t>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>IE listing</t>
+          <t>Kettle footprint area (cm²)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>https://www.currys.ie/ieen/household-appliances/small-kitchen-appliances/kettles/philips-daily-collection-hd9334-12-jug-kettle-white-blue-10164709-pdt.html</t>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>— (kettle L×D not confirmed)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Specs (capacity, power, voltage) — datasheet mirror</t>
+          <t>Cordless-base footprint</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>https://icecat.biz/en/p/philips/hd9334-90/daily+collection-electric+kettles-8710103809654-hd9334-90-35700663.html</t>
+          <t>N/A (corded travel — no separate base)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Dimensions (Philips datasheet PDF)</t>
+          <t>Footprint total (kettle+base)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>https://gzhls.at/blob/ldb/b/3/4/5/f7e120e5116fc98814833e52b29d019eee9b.pdf</t>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Philips Daily Collection HD9334/12 (1.5L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Filter / cordless / window / material</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+          <t>Power (W)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Dualit 1 Litre Jug Kettle 72200 (1L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Specs (capacity, min boil, dims, filter, material, warranty)</t>
+          <t>Boil time</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Dualit 1 Litre Jug Kettle 72200 (1L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Model number 72200</t>
+          <t>Corded/Cordless</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>https://www.hartsofstur.com/dualit-1-litre-mini-jug-kettle-chrome-72200.html</t>
+          <t>Corded</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Dualit 1 Litre Jug Kettle 72200 (1L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>IE category page</t>
+          <t>Voltage</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>https://www.currys.ie/appliances/small-kitchen-appliances/kettles/dualit</t>
+          <t>Dual / universal 120–240V</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Kenwood Discovery JKP250 (0.5L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Specs (capacity, power, voltage, filter, window, material, warranty)</t>
+          <t>Limescale filter</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Kenwood Discovery JKP250 (0.5L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>IE listing (Currys kettle category)</t>
+          <t>Noise / quiet boil</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>https://www.currys.ie/appliances/small-kitchen-appliances/kettles/kenwood</t>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Kenwood Discovery JKP250 (0.5L)</t>
+          <t>Russell Hobbs 0.85L</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Dimensions (UK retailer quoting Kenwood — verify)</t>
+          <t>Level window</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>https://maxwellselectrical.co.uk/kenwood-jkp250-100023951.html</t>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Russell Hobbs 0.85L</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Plastic</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Russell Hobbs 0.85L</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Warranty</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>2 years</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Russell Hobbs 0.85L</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Where sold in IE</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Amazon.ie; Harvey Norman.ie; Soundstore.ie (Currys.ie not confirmed)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/Russell-Hobbs-23840-Compact-Electric/dp/B07B96BQM6</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Russell Hobbs 0.85L</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Price (€) + date</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Amazon.ie €19.00 (RRP €24.99), 2026-06-15; HN.ie &amp; Soundstore.ie needs verification</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>partly confirmed — see value</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amazon.ie/Russell-Hobbs-23840-Compact-Electric/dp/B07B96BQM6</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Russell Hobbs 0.85L</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Cost/boil — power×time (€)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (no boil time published)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://ie.russellhobbs.com/product/travel-kettle-23840</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Russell Hobbs 0.85L</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Est. energy full boil (kWh)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>0.09329999999999999</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Russell Hobbs 0.85L</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Est. cost full boil (€)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>0.0339</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Russell Hobbs 0.85L</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Est. cost per cup (€, 0.25L)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Russell Hobbs 0.85L</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Affiliate network</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Amazon Associates (Amazon.ie); Awin (HN.ie)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>inference (no cited source)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Compact standard</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Capacity (L)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Cups per boil</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>— (derived: capacity ÷ 0.25 L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Min boil</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>1 cup / 0.3 L (markings 0.3/0.5/0.7/1.0 L)</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Can boil 1 cup?</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Yes (0.3 L)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Kettle dims L×D×H (cm)</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>16.6 × 20.0 × 23.2 cm (W×D×H)</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Kettle footprint L×D (cm)</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>16.6 × 20.0</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Kettle footprint area (cm²)</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>332</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>— (derived: L × D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Cordless-base footprint</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Footprint total (kettle+base)</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Power (W)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>2400</v>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Boil time</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>1 L from cold in 3 min 07 s (187 s) — full boil, published</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Corded/Cordless</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Cordless</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Voltage</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (220–240V expected)</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Limescale filter</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Noise / quiet boil</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Level window</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Plastic</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Warranty</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>2 years</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Where sold in IE</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (not confirmed on the 4 allowed stores; only Tefal IE shop)</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>— (not confirmed in an allowed IE store; Tefal IE shop only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Price (€) + date</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>needs verification on allowed store (Tefal IE shop €61.00, 2026-06-15, not an allowed source)</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>— (not confirmed in an allowed IE store; Tefal IE shop only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Cost/boil — power×time (€)</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Full 1 L: 2400W×187s = 0.1247 kWh → €0.045</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tefal.ie/Breakfast/Kettles/Tefal-Includeo-KI533840-Kettle-%E2%80%93-1L-Black/p/7211004563</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Est. energy full boil (kWh)</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="n">
+        <v>0.1098</v>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Est. cost full boil (€)</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>0.0399</v>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Est. cost per cup (€, 0.25L)</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Tefal 1L</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Affiliate network</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (no allowed IE retailer confirmed)</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>inference (no cited source)</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Standard jug (smallest Philips in IE)</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Capacity (L)</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Cups per boil</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>— (derived: capacity ÷ 0.25 L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Min boil</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Can boil 1 cup?</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Kettle dims L×D×H (cm)</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>22.3 × 16.2 × 25.4 cm</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Kettle footprint L×D (cm)</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>22.3 × 16.2</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Kettle footprint area (cm²)</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="n">
+        <v>361.3</v>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>— (derived: L × D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Cordless-base footprint</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Footprint total (kettle+base)</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Power (W)</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>2200</v>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Boil time</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Corded/Cordless</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Cordless</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Voltage</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>220–240V</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Limescale filter</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Yes (micro-mesh &gt;180 µm)</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Noise / quiet boil</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Level window</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Plastic (PP) + concealed steel element</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Warranty</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>2 years (variant needs verification)</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>partly confirmed — see value</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Where sold in IE</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Currys.ie (HN.ie stocks Philips; this model not confirmed)</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.currys.ie/ieen/household-appliances/small-kitchen-appliances/kettles/philips-daily-collection-hd9334-12-jug-kettle-white-blue-10164709-pdt.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Price (€) + date</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>needs verification on allowed store (ref ~€39 at non-allowed source, 2026-06-15)</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.currys.ie/ieen/household-appliances/small-kitchen-appliances/kettles/philips-daily-collection-hd9334-12-jug-kettle-white-blue-10164709-pdt.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Cost/boil — power×time (€)</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (no boil time published)</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.philips.com/c-p/HD9334_90R1/daily-collection-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Est. energy full boil (kWh)</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>0.1647</v>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Est. cost full boil (€)</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="n">
+        <v>0.0598</v>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Est. cost per cup (€, 0.25L)</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Philips 1.5L</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Affiliate network</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Awin (Currys.ie)</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>inference (no cited source)</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Compact standard</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Capacity (L)</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Cups per boil</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>— (derived: capacity ÷ 0.25 L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Min boil</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>2 cups (manufacturer minimum)</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Can boil 1 cup?</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>No (min 2 cups)</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Kettle dims L×D×H (cm)</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>20 × 16 × 23 cm (weight 0.92 kg)</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Kettle footprint L×D (cm)</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>20 × 16</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Kettle footprint area (cm²)</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>— (derived: L × D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Cordless-base footprint</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Footprint total (kettle+base)</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Power (W)</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (1L 72200 not stated; only the 1.5L 'Lite' is 3 kW — do not assume)</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Boil time</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Corded/Cordless</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Cordless</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Voltage</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (220–240V implied)</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>Limescale filter</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>Noise / quiet boil</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (no quiet-boil claim on the 1L model; Dualit markets the Classic as quiet, not this)</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>Level window</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Stainless steel</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Warranty</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>1 year (mfr; some retailers list 2–3)</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Where sold in IE</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Currys.ie (Dualit category page confirmed; exact 72200 product/price/stock needs verification)</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>partly confirmed — see value</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>https://www.currys.ie/appliances/small-kitchen-appliances/kettles/dualit</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Price (€) + date</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (Currys.ie / Amazon.ie not retrievable; 72200 not found in Amazon.ie search)</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.currys.ie/appliances/small-kitchen-appliances/kettles/dualit</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Cost/boil — power×time (€)</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (no boil time and no confirmed wattage)</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dualit.com/products/1-litre-jug-kettle</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Est. energy full boil (kWh)</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="n">
+        <v>0.1098</v>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Est. cost full boil (€)</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="n">
+        <v>0.0399</v>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Est. cost per cup (€, 0.25L)</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>Dualit 1L</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Affiliate network</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Awin (Currys.ie)</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>inference (no cited source)</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Travel / mini</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Capacity (L)</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Cups per boil</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>— (derived: capacity ÷ 0.25 L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Min boil</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>NV (ships with 2×200 ml cups; MIN marking not confirmed)</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Can boil 1 cup?</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Kettle dims L×D×H (cm)</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>16.8 × 9.8 × 17.0 cm (W×D×H)</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Kettle footprint L×D (cm)</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>16.8 × 9.8</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Kettle footprint area (cm²)</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="n">
+        <v>164.6</v>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>— (derived: L × D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Cordless-base footprint</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>N/A (corded travel — no separate base)</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Footprint total (kettle+base)</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>16.8 × 9.8 (kettle only)</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Power (W)</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="n">
+        <v>650</v>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Boil time</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Corded/Cordless</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Corded</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Voltage</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Dual / universal 120–240V</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Limescale filter</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Noise / quiet boil</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Level window</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Plastic</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Warranty</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Where sold in IE</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>Currys.ie (listed)</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>confirmed (mfr/retailer page, via search snippet)</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>https://www.currys.ie/appliances/small-kitchen-appliances/kettles/kenwood</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Price (€) + date</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (listed on Currys.ie; € not retrievable, 2026-06-15)</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.currys.ie/appliances/small-kitchen-appliances/kettles/kenwood</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Cost/boil — power×time (€)</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>needs verification (no boil time published)</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>needs verification</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kenwoodworld.com/en/s/JKP250</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Est. energy full boil (kWh)</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="n">
+        <v>0.0549</v>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>Est. cost full boil (€)</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="n">
+        <v>0.0199</v>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Est. cost per cup (€, 0.25L)</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>estimate (physics — see Method)</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>— (estimate; assumptions on Method sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>Kenwood 0.5L</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>Affiliate network</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>Awin (Currys.ie)</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>inference (no cited source)</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1698,290 +4872,262 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="112" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>COMPACT KETTLES — IRELAND · research data for roomnabs page #2</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Compiled 2026-06-15. 5 products (the two 1.7L 'quiet' jugs were dropped — see below). Rows on 'Kettles'; URLs on 'Sources'.</t>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Compiled 2026-06-15. 5 products. 'Kettles' = overview (one row each). 'Data &amp; sources' = one row per datum,</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr"/>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>with value + status + source URL side by side (so every data point sits next to its source).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>DATA RULES</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>• Nothing is invented or estimated. Unconfirmed values = 'needs verification' (NV).</t>
-        </is>
-      </c>
-    </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>• Nothing is invented or estimated (except the labelled physical-cost columns). Unconfirmed = 'needs verification'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>• Specs prefer the official manufacturer page; price/stock prefer Currys.ie / HarveyNorman.ie / Soundstore.ie / Amazon.ie.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>• No marketing prose — factual numbers/claims only. Manufacturer claim text is quoted verbatim where used.</t>
-        </is>
-      </c>
-    </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>• No marketing prose — factual numbers/claims only; manufacturer claim text quoted verbatim where used.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>IMPORTANT COLLECTION CAVEAT</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>• All manufacturer and retailer pages returned HTTP 403 to automated fetching, so values come from search-indexed</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  snippets attributed to those exact pages, not direct page reads. Fields not corroborable that way are marked NV.</t>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>• Every manufacturer and retailer page returned HTTP 403 to automated fetching, so values were read from search-indexed</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>• A human should open the cited pages in a normal browser to lock down live € prices, base footprints and any NV fields.</t>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  snippets attributed to those exact pages, not direct page reads. Status reads 'via search snippet' to reflect this.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>• Open the cited pages in a normal browser to lock down live € prices, base footprints and the 'needs verification' fields.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>FOOTPRINT (kettle + cordless base) — STATE PER PRODUCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>• Base footprint was NOT published by any manufacturer → 'needs verification' for all cordless models.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>• Full kettle+base footprint is complete for ONLY Kenwood JKP250 (corded travel → no separate base; total = kettle).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>• Tefal / Philips / Dualit: kettle footprint known, base NV → total NV. RH 23840: even kettle L×D is NV (height only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>ELECTRICITY TARIFF</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>• 0.363 €/kWh (Ireland, Jun 2026), reused from page #1 (air-fryer guide research).</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>• Corroborated by external 2026 sources (~35c/kWh incl. VAT): selectra.ie/energy/guides/electricity-prices-ireland;</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  saveonheat.ie/electricity-cost-per-kwh-ireland.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>CALCULATED FIELDS (labelled '(calc)')</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>• Cups per boil = capacity ÷ 0.25 L.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>• Kettle footprint area = L × D (cm²). Footprint rank is by this area, ascending. Cordless-base footprints were NOT</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  published for any model, so a true 'kettle + base' total is NV for the cordless models; ranking uses kettle footprint only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>COST PER BOIL — TWO METHODS, KEPT SEPARATE</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>• 'power × time' column: only where the manufacturer publishes a boil time. (W÷1000) × time(h) × tariff.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Confirmed full-boil time only for Tefal Includeo (1 L in 3:07 → €0.045).</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>• Estimate columns: physical energy to heat water from 15°C to 100°C at 90% efficiency × tariff.</t>
-        </is>
-      </c>
-    </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Factor = 4.186 kJ/(kg·K) × 85 K ÷ 3600 ÷ 0.9 = 0.10982 kWh per litre. Per cup (0.25 L) = €0.0100.</t>
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>• Estimate columns: energy to heat water 15°C→100°C at 90% efficiency × tariff.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  These are ESTIMATES (physics-based), not manufacturer specs — use as a like-for-like comparison only.</t>
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Factor = 4.186 × 85 ÷ 3600 ÷ 0.9 = 0.10982 kWh/L. Per cup (0.25 L) = €0.0100. ESTIMATES, not specs.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr"/>
+      <c r="A30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>REMOVED AT USER REQUEST</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>• Russell Hobbs Quiet Boil 20462 (1.7L) and Breville Edge VKT236 (1.7L) — both full-size 'quiet' jugs, NOT compact.</t>
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>• Russell Hobbs Quiet Boil 20462 (1.7L) and Breville Edge VKT236 (1.7L) — full-size 'quiet' jugs, NOT compact.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  No genuinely compact RH or Breville kettle is sold in the 4 allowed IE stores, so the 'compact quiet' niche was</t>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  No genuinely compact RH or Breville kettle is sold in the 4 allowed IE stores, so the niche was dropped, not padded.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  dropped rather than padded with 1.7L models.</t>
-        </is>
-      </c>
+      <c r="A34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr"/>
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>REMAINING FLAGS</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>REMAINING PRODUCT FLAGS</t>
+          <t>• Philips HD9334/12 (1.5L): smallest Philips in IE, kept as the higher-capacity option (not a 'quiet' model).</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>• Philips: NO travel/mini Philips in IE; whole range is 1.5–1.7L. Row uses the smallest (Daily HD9334/12, 1.5L,</t>
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>• Dualit chosen over Salter (no compact Salter in IE). Kenwood JKP250 chosen over Tower T10026 (not confirmed in IE).</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  borderline). It is NOT a 'quiet' model, so it was kept — say the word to drop it too.</t>
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>• Tefal Includeo (compact, boils 1 cup) NOT confirmed in the 4 allowed stores — verify on HN.ie / Amazon.ie before use.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>• Dualit chosen over Salter (Salter has no compact model in IE). Dualit 72200 is genuinely compact (1L); min boil = 2 cups.</t>
-        </is>
-      </c>
+      <c r="A39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>• Kenwood JKP250 chosen over Tower T10026 (Tower not confirmed in allowed IE stores).</t>
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>NET: genuinely compact + confirmed in an allowed IE store today = RH 23840 (travel), Kenwood JKP250 (travel),</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>• Tefal Includeo KI533840 is genuinely compact (1L, boils 1 cup) but was NOT confirmed in the 4 allowed stores</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  (only the Tefal IE manufacturer shop) — verify stock/price on HN.ie or Amazon.ie before using.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>NET: genuinely compact + confirmed in an allowed IE store today = RH 23840 (travel), Kenwood JKP250 (travel),</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>Dualit 72200 (compact). Tefal (compact) and Philips (borderline) need an allowed-store price/stock confirmation.</t>
         </is>

</xml_diff>